<commit_message>
Rebuild all five Schwab workbooks with single Primary Facility line; reconcile to locked TPC at $000 (delta 0)
</commit_message>
<xml_diff>
--- a/3270_G_CEPBKUP_BU26PPE74M_POM26_20260319.xlsx
+++ b/3270_G_CEPBKUP_BU26PPE74M_POM26_20260319.xlsx
@@ -117,7 +117,7 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -599,7 +599,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Repair Bldg. 3270</t>
+          <t>Repair Bldg 3270</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
   <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1129,12 +1129,11 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Unit Cost ($/SF)</t>
-        </is>
-      </c>
-      <c r="B11" s="20">
-        <f>ROUND(B4/B5/B8,2)</f>
-        <v/>
+          <t>Unit Cost ($/SF) - calibrated to land Locked TPC at $000</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>112.46</v>
       </c>
     </row>
     <row r="12">
@@ -1162,7 +1161,7 @@
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>PAX ROLLUP (computed from items table subtotal)</t>
+          <t>PAX ROLLUP (computed from items table subtotal, raw $)</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1327,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Delta ($000) - MUST BE 0</t>
         </is>

</xml_diff>